<commit_message>
Update master file inventory Excel and clean workspace scrap
</commit_message>
<xml_diff>
--- a/100_Beal_Street_Master_File_Inventory_v1.xlsx
+++ b/100_Beal_Street_Master_File_Inventory_v1.xlsx
@@ -625,7 +625,7 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Report Date: September 20, 2026  •  Location: Hingham, Plymouth County, MA  •  Zero Web Scrapes</t>
+          <t>Report Date: September 21, 2026  •  Location: Hingham, Plymouth County, MA  •  Zero Web Scrapes</t>
         </is>
       </c>
     </row>
@@ -1563,7 +1563,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: September 20, 2026 • Total Records: 311 • Zero Web Scrapes</t>
+          <t>Generated: September 21, 2026 • Total Records: 311 • Zero Web Scrapes</t>
         </is>
       </c>
     </row>
@@ -23450,7 +23450,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: September 20, 2026 • Total Records: 71 • Zero Web Scrapes</t>
+          <t>Generated: September 21, 2026 • Total Records: 71 • Zero Web Scrapes</t>
         </is>
       </c>
     </row>
@@ -28537,7 +28537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: September 20, 2026 • Total Records: 223 • Zero Web Scrapes</t>
+          <t>Generated: September 21, 2026 • Total Records: 223 • Zero Web Scrapes</t>
         </is>
       </c>
     </row>
@@ -44264,7 +44264,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: September 20, 2026 • Total Records: 16 • Zero Web Scrapes</t>
+          <t>Generated: September 21, 2026 • Total Records: 16 • Zero Web Scrapes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add standalone package folder for verifiable facts and supporting human documents v1
</commit_message>
<xml_diff>
--- a/100_Beal_Street_Master_File_Inventory_v1.xlsx
+++ b/100_Beal_Street_Master_File_Inventory_v1.xlsx
@@ -14,9 +14,9 @@
     <sheet name="Repository Index &amp; Governance" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Files Master Catalog'!$A$4:$N$319</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Files Master Catalog'!$A$4:$N$339</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Downloaded Sources'!$A$4:$N$75</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Agent Deliverables'!$A$4:$N$231</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Agent Deliverables'!$A$4:$N$251</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Repository Index &amp; Governance'!$A$4:$N$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:I44"/>
+  <dimension ref="B2:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -633,7 +633,7 @@
       <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Total Files Cataloged
-315</t>
+335</t>
         </is>
       </c>
       <c r="C6" s="5" t="n"/>
@@ -647,7 +647,7 @@
       <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Agent Deliverables
-227</t>
+247</t>
         </is>
       </c>
       <c r="G6" s="5" t="n"/>
@@ -954,7 +954,7 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>862.8 MB (904,748,272 bytes across 315 active verified files)</t>
+          <t>901.8 MB (945,600,477 bytes across 335 active verified files)</t>
         </is>
       </c>
       <c r="D25" s="9" t="n"/>
@@ -1013,20 +1013,20 @@
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>Companion Markdown Transcriptions</t>
+          <t>Agent Synthesized Work</t>
         </is>
       </c>
       <c r="D30" s="12" t="n">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>2.7 MB</t>
+          <t>39.0 MB</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>MD, PDF, ZIP</t>
         </is>
       </c>
       <c r="G30" s="8" t="inlineStr">
@@ -1045,20 +1045,20 @@
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>Detailed Timeline &amp; Plain-English TLDR</t>
+          <t>Companion Markdown Transcriptions</t>
         </is>
       </c>
       <c r="D31" s="12" t="n">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>154.7 KB</t>
+          <t>2.7 MB</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>MD, PDF</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
@@ -1077,15 +1077,15 @@
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>Executive Reports &amp; Briefings</t>
+          <t>Detailed Timeline &amp; Plain-English TLDR</t>
         </is>
       </c>
       <c r="D32" s="12" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>1.2 MB</t>
+          <t>154.7 KB</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
@@ -1109,15 +1109,15 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Master Chronological Compendiums</t>
+          <t>Executive Reports &amp; Briefings</t>
         </is>
       </c>
       <c r="D33" s="12" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>104.5 MB</t>
+          <t>1.2 MB</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Quality Control Audits</t>
+          <t>Master Chronological Compendiums</t>
         </is>
       </c>
       <c r="D34" s="12" t="n">
@@ -1149,12 +1149,12 @@
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>101.8 KB</t>
+          <t>104.5 MB</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>MD, PDF</t>
         </is>
       </c>
       <c r="G34" s="8" t="inlineStr">
@@ -1173,20 +1173,20 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Speech-to-Text Meeting Transcripts</t>
+          <t>Quality Control Audits</t>
         </is>
       </c>
       <c r="D35" s="12" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E35" s="12" t="inlineStr">
         <is>
-          <t>539.5 KB</t>
+          <t>101.8 KB</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
         <is>
-          <t>MD, TXT</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="G35" s="8" t="inlineStr">
@@ -1205,20 +1205,20 @@
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Video Presentations &amp; Narration Decks</t>
+          <t>Speech-to-Text Meeting Transcripts</t>
         </is>
       </c>
       <c r="D36" s="12" t="n">
-        <v>134</v>
+        <v>7</v>
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>358.6 MB</t>
+          <t>539.5 KB</t>
         </is>
       </c>
       <c r="F36" s="8" t="inlineStr">
         <is>
-          <t>HTML, JPG, MD, MP4, PDF, PNG, PPTX, TXT, VTT, WAV</t>
+          <t>MD, TXT</t>
         </is>
       </c>
       <c r="G36" s="8" t="inlineStr">
@@ -1237,20 +1237,20 @@
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>Visual Infographics &amp; Timelines</t>
+          <t>Video Presentations &amp; Narration Decks</t>
         </is>
       </c>
       <c r="D37" s="12" t="n">
-        <v>6</v>
+        <v>134</v>
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>3.5 MB</t>
+          <t>358.6 MB</t>
         </is>
       </c>
       <c r="F37" s="8" t="inlineStr">
         <is>
-          <t>JPG, PDF, PNG</t>
+          <t>HTML, JPG, MD, MP4, PDF, PNG, PPTX, TXT, VTT, WAV</t>
         </is>
       </c>
       <c r="G37" s="8" t="inlineStr">
@@ -1264,30 +1264,30 @@
     <row r="38">
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>Downloaded Primary Source</t>
+          <t>Agent-Created Deliverable</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Architectural &amp; Survey Plans</t>
+          <t>Visual Infographics &amp; Timelines</t>
         </is>
       </c>
       <c r="D38" s="12" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>67.0 MB</t>
+          <t>3.5 MB</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>JPG, PDF, WEBP</t>
+          <t>JPG, PDF, PNG</t>
         </is>
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
-          <t>Authentic primary municipal record</t>
+          <t>Synthesized briefing / report</t>
         </is>
       </c>
       <c r="H38" s="9" t="n"/>
@@ -1301,20 +1301,20 @@
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>Board Agendas &amp; Minutes (PDF)</t>
+          <t>Architectural &amp; Survey Plans</t>
         </is>
       </c>
       <c r="D39" s="12" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="E39" s="12" t="inlineStr">
         <is>
-          <t>3.1 MB</t>
+          <t>67.0 MB</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
-          <t>PDF</t>
+          <t>JPG, PDF, WEBP</t>
         </is>
       </c>
       <c r="G39" s="8" t="inlineStr">
@@ -1333,20 +1333,20 @@
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>Meeting Broadcast Audio (MP3)</t>
+          <t>Board Agendas &amp; Minutes (PDF)</t>
         </is>
       </c>
       <c r="D40" s="12" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>275.0 MB</t>
+          <t>3.1 MB</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t>MP3</t>
+          <t>PDF</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr">
@@ -1365,20 +1365,20 @@
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>Municipal Documents, Warrants &amp; Deeds</t>
+          <t>Meeting Broadcast Audio (MP3)</t>
         </is>
       </c>
       <c r="D41" s="12" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E41" s="12" t="inlineStr">
         <is>
-          <t>43.9 MB</t>
+          <t>275.0 MB</t>
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">
         <is>
-          <t>PDF</t>
+          <t>MP3</t>
         </is>
       </c>
       <c r="G41" s="8" t="inlineStr">
@@ -1397,20 +1397,20 @@
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>Registry Scans &amp; Recorded ORAD</t>
+          <t>Municipal Documents, Warrants &amp; Deeds</t>
         </is>
       </c>
       <c r="D42" s="12" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>2.0 MB</t>
+          <t>43.9 MB</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
-          <t>PDF, PNG, TXT</t>
+          <t>PDF</t>
         </is>
       </c>
       <c r="G42" s="8" t="inlineStr">
@@ -1424,30 +1424,30 @@
     <row r="43">
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>Master Compendium &amp; Archive</t>
+          <t>Downloaded Primary Source</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Authoritative Single-File Code &amp; Document Compendium</t>
+          <t>Registry Scans &amp; Recorded ORAD</t>
         </is>
       </c>
       <c r="D43" s="12" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
-          <t>511.4 KB</t>
+          <t>2.0 MB</t>
         </is>
       </c>
       <c r="F43" s="8" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>PDF, PNG, TXT</t>
         </is>
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
-          <t>Repository catalog</t>
+          <t>Authentic primary municipal record</t>
         </is>
       </c>
       <c r="H43" s="9" t="n"/>
@@ -1456,25 +1456,25 @@
     <row r="44">
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>Repository Documentation &amp; Index</t>
+          <t>Master Compendium &amp; Archive</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>Repository Index &amp; Governance</t>
+          <t>Authoritative Single-File Code &amp; Document Compendium</t>
         </is>
       </c>
       <c r="D44" s="12" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>205.2 KB</t>
+          <t>511.4 KB</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
         <is>
-          <t>JSON, MD</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="G44" s="8" t="inlineStr">
@@ -1485,8 +1485,40 @@
       <c r="H44" s="9" t="n"/>
       <c r="I44" s="10" t="n"/>
     </row>
+    <row r="45">
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>Repository Documentation &amp; Index</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Repository Index &amp; Governance</t>
+        </is>
+      </c>
+      <c r="D45" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="E45" s="12" t="inlineStr">
+        <is>
+          <t>205.2 KB</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>JSON, MD</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>Repository catalog</t>
+        </is>
+      </c>
+      <c r="H45" s="9" t="n"/>
+      <c r="I45" s="10" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="36">
+  <mergeCells count="37">
     <mergeCell ref="G38:I38"/>
     <mergeCell ref="C23:I23"/>
     <mergeCell ref="C17:I17"/>
@@ -1498,6 +1530,7 @@
     <mergeCell ref="G33:I33"/>
     <mergeCell ref="C13:I13"/>
     <mergeCell ref="C18:I18"/>
+    <mergeCell ref="G45:I45"/>
     <mergeCell ref="G35:I35"/>
     <mergeCell ref="C24:I24"/>
     <mergeCell ref="C15:I15"/>
@@ -1534,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N319"/>
+  <dimension ref="A1:N339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1563,7 +1596,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: September 22, 2026 • Total Records: 315 • Zero Web Scrapes</t>
+          <t>Generated: September 22, 2026 • Total Records: 335 • Zero Web Scrapes</t>
         </is>
       </c>
     </row>
@@ -23689,8 +23722,1408 @@
         </is>
       </c>
     </row>
+    <row r="320">
+      <c r="A320" s="19" t="inlineStr">
+        <is>
+          <t>FL-316</t>
+        </is>
+      </c>
+      <c r="B320" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C320" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D320" s="20" t="inlineStr">
+        <is>
+          <t>100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1.zip</t>
+        </is>
+      </c>
+      <c r="E320" s="19" t="inlineStr">
+        <is>
+          <t>ZIP</t>
+        </is>
+      </c>
+      <c r="F320" s="21" t="n">
+        <v>19847898</v>
+      </c>
+      <c r="G320" s="22" t="inlineStr">
+        <is>
+          <t>18.9 MB</t>
+        </is>
+      </c>
+      <c r="H320" s="19" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I320" s="20" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J320" s="20" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K320" s="23" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L320" s="19" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M320" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-22 09:14</t>
+        </is>
+      </c>
+      <c r="N320" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1.zip</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="15" t="inlineStr">
+        <is>
+          <t>FL-317</t>
+        </is>
+      </c>
+      <c r="B321" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C321" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D321" s="16" t="inlineStr">
+        <is>
+          <t>README_PACKAGE_v1.md</t>
+        </is>
+      </c>
+      <c r="E321" s="15" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="F321" s="17" t="n">
+        <v>5931</v>
+      </c>
+      <c r="G321" s="12" t="inlineStr">
+        <is>
+          <t>5.8 KB</t>
+        </is>
+      </c>
+      <c r="H321" s="15" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I321" s="16" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J321" s="16" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K321" s="18" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L321" s="15" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M321" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-22 09:14</t>
+        </is>
+      </c>
+      <c r="N321" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/README_PACKAGE_v1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="19" t="inlineStr">
+        <is>
+          <t>FL-318</t>
+        </is>
+      </c>
+      <c r="B322" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C322" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D322" s="20" t="inlineStr">
+        <is>
+          <t>01_100_Beal_Street_Verifiable_Facts_and_Human_Document_v1.md</t>
+        </is>
+      </c>
+      <c r="E322" s="19" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="F322" s="21" t="n">
+        <v>22221</v>
+      </c>
+      <c r="G322" s="22" t="inlineStr">
+        <is>
+          <t>21.7 KB</t>
+        </is>
+      </c>
+      <c r="H322" s="19" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I322" s="20" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J322" s="20" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K322" s="23" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L322" s="19" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M322" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-22 09:10</t>
+        </is>
+      </c>
+      <c r="N322" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/01_Executive_and_Human_Documents/01_100_Beal_Street_Verifiable_Facts_and_Human_Document_v1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="15" t="inlineStr">
+        <is>
+          <t>FL-319</t>
+        </is>
+      </c>
+      <c r="B323" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C323" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D323" s="16" t="inlineStr">
+        <is>
+          <t>01_100_Beal_Street_Verifiable_Facts_and_Human_Document_v1.pdf</t>
+        </is>
+      </c>
+      <c r="E323" s="15" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F323" s="17" t="n">
+        <v>103490</v>
+      </c>
+      <c r="G323" s="12" t="inlineStr">
+        <is>
+          <t>101.1 KB</t>
+        </is>
+      </c>
+      <c r="H323" s="15" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I323" s="16" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J323" s="16" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K323" s="18" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L323" s="15" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M323" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-22 09:10</t>
+        </is>
+      </c>
+      <c r="N323" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/01_Executive_and_Human_Documents/01_100_Beal_Street_Verifiable_Facts_and_Human_Document_v1.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="19" t="inlineStr">
+        <is>
+          <t>FL-320</t>
+        </is>
+      </c>
+      <c r="B324" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C324" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D324" s="20" t="inlineStr">
+        <is>
+          <t>02_100_Beal_Street_Records_Verification_Checklist_and_Audit_v1.md</t>
+        </is>
+      </c>
+      <c r="E324" s="19" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="F324" s="21" t="n">
+        <v>28047</v>
+      </c>
+      <c r="G324" s="22" t="inlineStr">
+        <is>
+          <t>27.4 KB</t>
+        </is>
+      </c>
+      <c r="H324" s="19" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I324" s="20" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J324" s="20" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K324" s="23" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L324" s="19" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M324" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-22 09:06</t>
+        </is>
+      </c>
+      <c r="N324" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/01_Executive_and_Human_Documents/02_100_Beal_Street_Records_Verification_Checklist_and_Audit_v1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="15" t="inlineStr">
+        <is>
+          <t>FL-321</t>
+        </is>
+      </c>
+      <c r="B325" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C325" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D325" s="16" t="inlineStr">
+        <is>
+          <t>02_100_Beal_Street_Records_Verification_Checklist_and_Audit_v1.pdf</t>
+        </is>
+      </c>
+      <c r="E325" s="15" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F325" s="17" t="n">
+        <v>132623</v>
+      </c>
+      <c r="G325" s="12" t="inlineStr">
+        <is>
+          <t>129.5 KB</t>
+        </is>
+      </c>
+      <c r="H325" s="15" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I325" s="16" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J325" s="16" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K325" s="18" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L325" s="15" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M325" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-22 09:08</t>
+        </is>
+      </c>
+      <c r="N325" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/01_Executive_and_Human_Documents/02_100_Beal_Street_Records_Verification_Checklist_and_Audit_v1.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="19" t="inlineStr">
+        <is>
+          <t>FL-322</t>
+        </is>
+      </c>
+      <c r="B326" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C326" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D326" s="20" t="inlineStr">
+        <is>
+          <t>03_100_Beal_Street_The_True_Story_and_Evidence_v1.md</t>
+        </is>
+      </c>
+      <c r="E326" s="19" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="F326" s="21" t="n">
+        <v>12031</v>
+      </c>
+      <c r="G326" s="22" t="inlineStr">
+        <is>
+          <t>11.7 KB</t>
+        </is>
+      </c>
+      <c r="H326" s="19" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I326" s="20" t="inlineStr">
+        <is>
+          <t>Primary Municipal Records &amp; Educational Architecture</t>
+        </is>
+      </c>
+      <c r="J326" s="20" t="inlineStr">
+        <is>
+          <t>M.G.L. c. 121B; M.G.L. c. 184A; M.G.L. c. 44, § 7; Plymouth Registry Instruments</t>
+        </is>
+      </c>
+      <c r="K326" s="23" t="inlineStr">
+        <is>
+          <t>Dedicated 2-page educational guide and evidence ledger for family and community members. Page 1 provides a 1-page unspun narrative essay; Page 2 provides the companion Works Cited mapping every point to primary documents with repository file names.</t>
+        </is>
+      </c>
+      <c r="L326" s="19" t="inlineStr">
+        <is>
+          <t>Community Educational Guide &amp; Evidence Ledger (Verified)</t>
+        </is>
+      </c>
+      <c r="M326" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:27</t>
+        </is>
+      </c>
+      <c r="N326" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/01_Executive_and_Human_Documents/03_100_Beal_Street_The_True_Story_and_Evidence_v1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="15" t="inlineStr">
+        <is>
+          <t>FL-323</t>
+        </is>
+      </c>
+      <c r="B327" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C327" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D327" s="16" t="inlineStr">
+        <is>
+          <t>03_100_Beal_Street_The_True_Story_and_Evidence_v1.pdf</t>
+        </is>
+      </c>
+      <c r="E327" s="15" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F327" s="17" t="n">
+        <v>74343</v>
+      </c>
+      <c r="G327" s="12" t="inlineStr">
+        <is>
+          <t>72.6 KB</t>
+        </is>
+      </c>
+      <c r="H327" s="15" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I327" s="16" t="inlineStr">
+        <is>
+          <t>Primary Municipal Records &amp; Educational Architecture</t>
+        </is>
+      </c>
+      <c r="J327" s="16" t="inlineStr">
+        <is>
+          <t>M.G.L. c. 121B; M.G.L. c. 184A; M.G.L. c. 44, § 7; Plymouth Registry Instruments</t>
+        </is>
+      </c>
+      <c r="K327" s="18" t="inlineStr">
+        <is>
+          <t>Dedicated 2-page educational guide and evidence ledger for family and community members. Page 1 provides a 1-page unspun narrative essay; Page 2 provides the companion Works Cited mapping every point to primary documents with repository file names.</t>
+        </is>
+      </c>
+      <c r="L327" s="15" t="inlineStr">
+        <is>
+          <t>Community Educational Guide &amp; Evidence Ledger (Verified)</t>
+        </is>
+      </c>
+      <c r="M327" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:27</t>
+        </is>
+      </c>
+      <c r="N327" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/01_Executive_and_Human_Documents/03_100_Beal_Street_The_True_Story_and_Evidence_v1.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="19" t="inlineStr">
+        <is>
+          <t>FL-324</t>
+        </is>
+      </c>
+      <c r="B328" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C328" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D328" s="20" t="inlineStr">
+        <is>
+          <t>04_100_Beal_Street_Town_vs_HHA_Legal_Chronology_and_Minutes_v2.md</t>
+        </is>
+      </c>
+      <c r="E328" s="19" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="F328" s="21" t="n">
+        <v>31676</v>
+      </c>
+      <c r="G328" s="22" t="inlineStr">
+        <is>
+          <t>30.9 KB</t>
+        </is>
+      </c>
+      <c r="H328" s="19" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="I328" s="20" t="inlineStr">
+        <is>
+          <t>Primary Municipal Records / Mass. Registry of Deeds</t>
+        </is>
+      </c>
+      <c r="J328" s="20" t="inlineStr">
+        <is>
+          <t>Historical M.G.L. c. 184A, § 3; M.G.L. c. 184, § 23; M.G.L. c. 121B, § 34; Book 09097 Pg 158; Book 51379 Pg 244</t>
+        </is>
+      </c>
+      <c r="K328" s="23" t="inlineStr">
+        <is>
+          <t>Preliminary primary-source research chronology and record index; strictly neutral factual reporting; segregates verified facts, factual inferences, and open legal questions; includes missing documents inventory and disclaimer. Not a title opinion.</t>
+        </is>
+      </c>
+      <c r="L328" s="19" t="inlineStr">
+        <is>
+          <t>Neutral Primary Source Research Index &amp; Inventory (Verified)</t>
+        </is>
+      </c>
+      <c r="M328" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-17 09:44</t>
+        </is>
+      </c>
+      <c r="N328" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/01_Executive_and_Human_Documents/04_100_Beal_Street_Town_vs_HHA_Legal_Chronology_and_Minutes_v2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="15" t="inlineStr">
+        <is>
+          <t>FL-325</t>
+        </is>
+      </c>
+      <c r="B329" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C329" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D329" s="16" t="inlineStr">
+        <is>
+          <t>04_100_Beal_Street_Town_vs_HHA_Legal_Chronology_and_Minutes_v2.pdf</t>
+        </is>
+      </c>
+      <c r="E329" s="15" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F329" s="17" t="n">
+        <v>119536</v>
+      </c>
+      <c r="G329" s="12" t="inlineStr">
+        <is>
+          <t>116.7 KB</t>
+        </is>
+      </c>
+      <c r="H329" s="15" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="I329" s="16" t="inlineStr">
+        <is>
+          <t>Primary Municipal Records / Mass. Registry of Deeds</t>
+        </is>
+      </c>
+      <c r="J329" s="16" t="inlineStr">
+        <is>
+          <t>Historical M.G.L. c. 184A, § 3; M.G.L. c. 184, § 23; M.G.L. c. 121B, § 34; Book 09097 Pg 158; Book 51379 Pg 244</t>
+        </is>
+      </c>
+      <c r="K329" s="18" t="inlineStr">
+        <is>
+          <t>Preliminary primary-source research chronology and record index; strictly neutral factual reporting; segregates verified facts, factual inferences, and open legal questions; includes missing documents inventory and disclaimer. Not a title opinion.</t>
+        </is>
+      </c>
+      <c r="L329" s="15" t="inlineStr">
+        <is>
+          <t>Neutral Primary Source Research Index &amp; Inventory (Verified)</t>
+        </is>
+      </c>
+      <c r="M329" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-17 09:44</t>
+        </is>
+      </c>
+      <c r="N329" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/01_Executive_and_Human_Documents/04_100_Beal_Street_Town_vs_HHA_Legal_Chronology_and_Minutes_v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="19" t="inlineStr">
+        <is>
+          <t>FL-326</t>
+        </is>
+      </c>
+      <c r="B330" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C330" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D330" s="20" t="inlineStr">
+        <is>
+          <t>Exhibit_01_1989_Fee_Deed_and_ZBA_Decision_Bk09097_Pg158.pdf</t>
+        </is>
+      </c>
+      <c r="E330" s="19" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F330" s="21" t="n">
+        <v>228302</v>
+      </c>
+      <c r="G330" s="22" t="inlineStr">
+        <is>
+          <t>223.0 KB</t>
+        </is>
+      </c>
+      <c r="H330" s="19" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I330" s="20" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J330" s="20" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K330" s="23" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L330" s="19" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M330" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-14 09:24</t>
+        </is>
+      </c>
+      <c r="N330" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_01_1989_Fee_Deed_and_ZBA_Decision_Bk09097_Pg158.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="15" t="inlineStr">
+        <is>
+          <t>FL-327</t>
+        </is>
+      </c>
+      <c r="B331" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C331" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D331" s="16" t="inlineStr">
+        <is>
+          <t>Exhibit_02_2001_Gale_Subdivision_Plan_and_2024_ALTA_Survey.pdf</t>
+        </is>
+      </c>
+      <c r="E331" s="15" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F331" s="17" t="n">
+        <v>2390635</v>
+      </c>
+      <c r="G331" s="12" t="inlineStr">
+        <is>
+          <t>2.3 MB</t>
+        </is>
+      </c>
+      <c r="H331" s="15" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I331" s="16" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J331" s="16" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K331" s="18" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L331" s="15" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M331" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14 09:24</t>
+        </is>
+      </c>
+      <c r="N331" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_02_2001_Gale_Subdivision_Plan_and_2024_ALTA_Survey.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="19" t="inlineStr">
+        <is>
+          <t>FL-328</t>
+        </is>
+      </c>
+      <c r="B332" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C332" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D332" s="20" t="inlineStr">
+        <is>
+          <t>Exhibit_03_2006_Town_Meeting_Article_38_Certified_Vote.pdf</t>
+        </is>
+      </c>
+      <c r="E332" s="19" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F332" s="21" t="n">
+        <v>217985</v>
+      </c>
+      <c r="G332" s="22" t="inlineStr">
+        <is>
+          <t>212.9 KB</t>
+        </is>
+      </c>
+      <c r="H332" s="19" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I332" s="20" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J332" s="20" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K332" s="23" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L332" s="19" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M332" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-14 09:24</t>
+        </is>
+      </c>
+      <c r="N332" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_03_2006_Town_Meeting_Article_38_Certified_Vote.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="15" t="inlineStr">
+        <is>
+          <t>FL-329</t>
+        </is>
+      </c>
+      <c r="B333" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C333" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D333" s="16" t="inlineStr">
+        <is>
+          <t>Exhibit_04_2019_Select_Board_Executive_Session_Minutes_Lawsuit_Vote.pdf</t>
+        </is>
+      </c>
+      <c r="E333" s="15" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F333" s="17" t="n">
+        <v>50677</v>
+      </c>
+      <c r="G333" s="12" t="inlineStr">
+        <is>
+          <t>49.5 KB</t>
+        </is>
+      </c>
+      <c r="H333" s="15" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I333" s="16" t="inlineStr">
+        <is>
+          <t>Hingham Board of Selectmen (Healey, Power, Johnson)</t>
+        </is>
+      </c>
+      <c r="J333" s="16" t="inlineStr">
+        <is>
+          <t>M.G.L. c. 30A, § 21(a)(3) (Executive Session Litigation)</t>
+        </is>
+      </c>
+      <c r="K333" s="18" t="inlineStr">
+        <is>
+          <t>Executive Session minutes of Feb 26, 2019 recording 3-0 vote to file litigation against HHA to enforce 2001 MOU 9 days before 30-yr reverter expiration.</t>
+        </is>
+      </c>
+      <c r="L333" s="15" t="inlineStr">
+        <is>
+          <t>Official Municipal Minutes (Verified)</t>
+        </is>
+      </c>
+      <c r="M333" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14 08:38</t>
+        </is>
+      </c>
+      <c r="N333" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_04_2019_Select_Board_Executive_Session_Minutes_Lawsuit_Vote.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="19" t="inlineStr">
+        <is>
+          <t>FL-330</t>
+        </is>
+      </c>
+      <c r="B334" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C334" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D334" s="20" t="inlineStr">
+        <is>
+          <t>Exhibit_05_2019_HHA_Minutes_School_Tract_II_DHCD_Intervention.pdf</t>
+        </is>
+      </c>
+      <c r="E334" s="19" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F334" s="21" t="n">
+        <v>41327</v>
+      </c>
+      <c r="G334" s="22" t="inlineStr">
+        <is>
+          <t>40.4 KB</t>
+        </is>
+      </c>
+      <c r="H334" s="19" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I334" s="20" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J334" s="20" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K334" s="23" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L334" s="19" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M334" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-14 09:13</t>
+        </is>
+      </c>
+      <c r="N334" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_05_2019_HHA_Minutes_School_Tract_II_DHCD_Intervention.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="15" t="inlineStr">
+        <is>
+          <t>FL-331</t>
+        </is>
+      </c>
+      <c r="B335" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C335" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D335" s="16" t="inlineStr">
+        <is>
+          <t>Exhibit_06_2021_HHA_Minutes_4-0_Rescission_Vote.pdf</t>
+        </is>
+      </c>
+      <c r="E335" s="15" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F335" s="17" t="n">
+        <v>101165</v>
+      </c>
+      <c r="G335" s="12" t="inlineStr">
+        <is>
+          <t>98.8 KB</t>
+        </is>
+      </c>
+      <c r="H335" s="15" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I335" s="16" t="inlineStr">
+        <is>
+          <t>Hingham Housing Authority (Dir. James Marathas)</t>
+        </is>
+      </c>
+      <c r="J335" s="16" t="inlineStr">
+        <is>
+          <t>M.G.L. c. 121B, § 34; HHA By-Laws</t>
+        </is>
+      </c>
+      <c r="K335" s="18" t="inlineStr">
+        <is>
+          <t>Official meeting minutes of Sept 7, 2021 recording 4-0 vote formally rescinding the June 5, 2019 transfer motion, keeping land in HHA ownership.</t>
+        </is>
+      </c>
+      <c r="L335" s="15" t="inlineStr">
+        <is>
+          <t>Official Board Minutes (Verified)</t>
+        </is>
+      </c>
+      <c r="M335" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:46</t>
+        </is>
+      </c>
+      <c r="N335" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_06_2021_HHA_Minutes_4-0_Rescission_Vote.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="19" t="inlineStr">
+        <is>
+          <t>FL-332</t>
+        </is>
+      </c>
+      <c r="B336" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C336" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D336" s="20" t="inlineStr">
+        <is>
+          <t>Exhibit_07_2024_MassDEP_Recorded_ORAD_Bk59527_Pg273.pdf</t>
+        </is>
+      </c>
+      <c r="E336" s="19" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F336" s="21" t="n">
+        <v>468709</v>
+      </c>
+      <c r="G336" s="22" t="inlineStr">
+        <is>
+          <t>457.7 KB</t>
+        </is>
+      </c>
+      <c r="H336" s="19" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I336" s="20" t="inlineStr">
+        <is>
+          <t>Hingham Conservation Commission / MassDEP</t>
+        </is>
+      </c>
+      <c r="J336" s="20" t="inlineStr">
+        <is>
+          <t>Plymouth County Registry of Deeds Book 59527, Page 273 (Doc #78968)</t>
+        </is>
+      </c>
+      <c r="K336" s="23" t="inlineStr">
+        <is>
+          <t>Recorded Order of Resource Area Delineation (ORAD) WPA Form 4B officially approving wetland boundary lines on Dec 10, 2024.</t>
+        </is>
+      </c>
+      <c r="L336" s="19" t="inlineStr">
+        <is>
+          <t>Recorded Order (Verified)</t>
+        </is>
+      </c>
+      <c r="M336" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-15 15:26</t>
+        </is>
+      </c>
+      <c r="N336" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_07_2024_MassDEP_Recorded_ORAD_Bk59527_Pg273.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="15" t="inlineStr">
+        <is>
+          <t>FL-333</t>
+        </is>
+      </c>
+      <c r="B337" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C337" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D337" s="16" t="inlineStr">
+        <is>
+          <t>Exhibit_08_2025_HHA_Developer_RFP_155_Pages.pdf</t>
+        </is>
+      </c>
+      <c r="E337" s="15" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F337" s="17" t="n">
+        <v>13909202</v>
+      </c>
+      <c r="G337" s="12" t="inlineStr">
+        <is>
+          <t>13.3 MB</t>
+        </is>
+      </c>
+      <c r="H337" s="15" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I337" s="16" t="inlineStr">
+        <is>
+          <t>Hingham Housing Authority (James Marathas, ED)</t>
+        </is>
+      </c>
+      <c r="J337" s="16" t="inlineStr">
+        <is>
+          <t>M.G.L. c. 30B, § 16; M.G.L. c. 121B</t>
+        </is>
+      </c>
+      <c r="K337" s="18" t="inlineStr">
+        <is>
+          <t>Official 155-page Developer RFP package including Bohler engineering study, Lucas wetlands report, Control Point boundary survey, and draft 99-year ground lease.</t>
+        </is>
+      </c>
+      <c r="L337" s="15" t="inlineStr">
+        <is>
+          <t>Authentic Public RFP (Verified)</t>
+        </is>
+      </c>
+      <c r="M337" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14 09:20</t>
+        </is>
+      </c>
+      <c r="N337" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_08_2025_HHA_Developer_RFP_155_Pages.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="19" t="inlineStr">
+        <is>
+          <t>FL-334</t>
+        </is>
+      </c>
+      <c r="B338" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C338" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D338" s="20" t="inlineStr">
+        <is>
+          <t>Exhibit_09_2025_HHA_Minutes_Peabody_Developer_Award_Vote.pdf</t>
+        </is>
+      </c>
+      <c r="E338" s="19" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F338" s="21" t="n">
+        <v>107708</v>
+      </c>
+      <c r="G338" s="22" t="inlineStr">
+        <is>
+          <t>105.2 KB</t>
+        </is>
+      </c>
+      <c r="H338" s="19" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I338" s="20" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J338" s="20" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K338" s="23" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L338" s="19" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M338" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:46</t>
+        </is>
+      </c>
+      <c r="N338" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_09_2025_HHA_Minutes_Peabody_Developer_Award_Vote.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="15" t="inlineStr">
+        <is>
+          <t>FL-335</t>
+        </is>
+      </c>
+      <c r="B339" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C339" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D339" s="16" t="inlineStr">
+        <is>
+          <t>Exhibit_10_2026_Town_Meeting_Warrant_Article_12_CAL_Debt_Defeat.pdf</t>
+        </is>
+      </c>
+      <c r="E339" s="15" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F339" s="17" t="n">
+        <v>2958699</v>
+      </c>
+      <c r="G339" s="12" t="inlineStr">
+        <is>
+          <t>2.8 MB</t>
+        </is>
+      </c>
+      <c r="H339" s="15" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I339" s="16" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J339" s="16" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K339" s="18" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L339" s="15" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M339" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14 09:19</t>
+        </is>
+      </c>
+      <c r="N339" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_10_2026_Town_Meeting_Warrant_Article_12_CAL_Debt_Defeat.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:N319"/>
+  <autoFilter ref="A4:N339"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -28788,7 +30221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N231"/>
+  <dimension ref="A1:N251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -28817,7 +30250,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: September 22, 2026 • Total Records: 227 • Zero Web Scrapes</t>
+          <t>Generated: September 22, 2026 • Total Records: 247 • Zero Web Scrapes</t>
         </is>
       </c>
     </row>
@@ -44783,8 +46216,1408 @@
         </is>
       </c>
     </row>
+    <row r="232">
+      <c r="A232" s="19" t="inlineStr">
+        <is>
+          <t>FL-316</t>
+        </is>
+      </c>
+      <c r="B232" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C232" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D232" s="20" t="inlineStr">
+        <is>
+          <t>100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1.zip</t>
+        </is>
+      </c>
+      <c r="E232" s="19" t="inlineStr">
+        <is>
+          <t>ZIP</t>
+        </is>
+      </c>
+      <c r="F232" s="21" t="n">
+        <v>19847898</v>
+      </c>
+      <c r="G232" s="22" t="inlineStr">
+        <is>
+          <t>18.9 MB</t>
+        </is>
+      </c>
+      <c r="H232" s="19" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I232" s="20" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J232" s="20" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K232" s="23" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L232" s="19" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M232" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-22 09:14</t>
+        </is>
+      </c>
+      <c r="N232" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1.zip</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="15" t="inlineStr">
+        <is>
+          <t>FL-317</t>
+        </is>
+      </c>
+      <c r="B233" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C233" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D233" s="16" t="inlineStr">
+        <is>
+          <t>README_PACKAGE_v1.md</t>
+        </is>
+      </c>
+      <c r="E233" s="15" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="F233" s="17" t="n">
+        <v>5931</v>
+      </c>
+      <c r="G233" s="12" t="inlineStr">
+        <is>
+          <t>5.8 KB</t>
+        </is>
+      </c>
+      <c r="H233" s="15" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I233" s="16" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J233" s="16" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K233" s="18" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L233" s="15" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M233" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-22 09:14</t>
+        </is>
+      </c>
+      <c r="N233" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/README_PACKAGE_v1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="19" t="inlineStr">
+        <is>
+          <t>FL-318</t>
+        </is>
+      </c>
+      <c r="B234" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C234" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D234" s="20" t="inlineStr">
+        <is>
+          <t>01_100_Beal_Street_Verifiable_Facts_and_Human_Document_v1.md</t>
+        </is>
+      </c>
+      <c r="E234" s="19" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="F234" s="21" t="n">
+        <v>22221</v>
+      </c>
+      <c r="G234" s="22" t="inlineStr">
+        <is>
+          <t>21.7 KB</t>
+        </is>
+      </c>
+      <c r="H234" s="19" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I234" s="20" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J234" s="20" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K234" s="23" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L234" s="19" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M234" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-22 09:10</t>
+        </is>
+      </c>
+      <c r="N234" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/01_Executive_and_Human_Documents/01_100_Beal_Street_Verifiable_Facts_and_Human_Document_v1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="15" t="inlineStr">
+        <is>
+          <t>FL-319</t>
+        </is>
+      </c>
+      <c r="B235" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C235" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D235" s="16" t="inlineStr">
+        <is>
+          <t>01_100_Beal_Street_Verifiable_Facts_and_Human_Document_v1.pdf</t>
+        </is>
+      </c>
+      <c r="E235" s="15" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F235" s="17" t="n">
+        <v>103490</v>
+      </c>
+      <c r="G235" s="12" t="inlineStr">
+        <is>
+          <t>101.1 KB</t>
+        </is>
+      </c>
+      <c r="H235" s="15" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I235" s="16" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J235" s="16" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K235" s="18" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L235" s="15" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M235" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-22 09:10</t>
+        </is>
+      </c>
+      <c r="N235" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/01_Executive_and_Human_Documents/01_100_Beal_Street_Verifiable_Facts_and_Human_Document_v1.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="19" t="inlineStr">
+        <is>
+          <t>FL-320</t>
+        </is>
+      </c>
+      <c r="B236" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C236" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D236" s="20" t="inlineStr">
+        <is>
+          <t>02_100_Beal_Street_Records_Verification_Checklist_and_Audit_v1.md</t>
+        </is>
+      </c>
+      <c r="E236" s="19" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="F236" s="21" t="n">
+        <v>28047</v>
+      </c>
+      <c r="G236" s="22" t="inlineStr">
+        <is>
+          <t>27.4 KB</t>
+        </is>
+      </c>
+      <c r="H236" s="19" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I236" s="20" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J236" s="20" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K236" s="23" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L236" s="19" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M236" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-22 09:06</t>
+        </is>
+      </c>
+      <c r="N236" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/01_Executive_and_Human_Documents/02_100_Beal_Street_Records_Verification_Checklist_and_Audit_v1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="15" t="inlineStr">
+        <is>
+          <t>FL-321</t>
+        </is>
+      </c>
+      <c r="B237" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C237" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D237" s="16" t="inlineStr">
+        <is>
+          <t>02_100_Beal_Street_Records_Verification_Checklist_and_Audit_v1.pdf</t>
+        </is>
+      </c>
+      <c r="E237" s="15" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F237" s="17" t="n">
+        <v>132623</v>
+      </c>
+      <c r="G237" s="12" t="inlineStr">
+        <is>
+          <t>129.5 KB</t>
+        </is>
+      </c>
+      <c r="H237" s="15" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I237" s="16" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J237" s="16" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K237" s="18" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L237" s="15" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M237" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-22 09:08</t>
+        </is>
+      </c>
+      <c r="N237" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/01_Executive_and_Human_Documents/02_100_Beal_Street_Records_Verification_Checklist_and_Audit_v1.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="19" t="inlineStr">
+        <is>
+          <t>FL-322</t>
+        </is>
+      </c>
+      <c r="B238" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C238" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D238" s="20" t="inlineStr">
+        <is>
+          <t>03_100_Beal_Street_The_True_Story_and_Evidence_v1.md</t>
+        </is>
+      </c>
+      <c r="E238" s="19" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="F238" s="21" t="n">
+        <v>12031</v>
+      </c>
+      <c r="G238" s="22" t="inlineStr">
+        <is>
+          <t>11.7 KB</t>
+        </is>
+      </c>
+      <c r="H238" s="19" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I238" s="20" t="inlineStr">
+        <is>
+          <t>Primary Municipal Records &amp; Educational Architecture</t>
+        </is>
+      </c>
+      <c r="J238" s="20" t="inlineStr">
+        <is>
+          <t>M.G.L. c. 121B; M.G.L. c. 184A; M.G.L. c. 44, § 7; Plymouth Registry Instruments</t>
+        </is>
+      </c>
+      <c r="K238" s="23" t="inlineStr">
+        <is>
+          <t>Dedicated 2-page educational guide and evidence ledger for family and community members. Page 1 provides a 1-page unspun narrative essay; Page 2 provides the companion Works Cited mapping every point to primary documents with repository file names.</t>
+        </is>
+      </c>
+      <c r="L238" s="19" t="inlineStr">
+        <is>
+          <t>Community Educational Guide &amp; Evidence Ledger (Verified)</t>
+        </is>
+      </c>
+      <c r="M238" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:27</t>
+        </is>
+      </c>
+      <c r="N238" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/01_Executive_and_Human_Documents/03_100_Beal_Street_The_True_Story_and_Evidence_v1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="15" t="inlineStr">
+        <is>
+          <t>FL-323</t>
+        </is>
+      </c>
+      <c r="B239" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C239" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D239" s="16" t="inlineStr">
+        <is>
+          <t>03_100_Beal_Street_The_True_Story_and_Evidence_v1.pdf</t>
+        </is>
+      </c>
+      <c r="E239" s="15" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F239" s="17" t="n">
+        <v>74343</v>
+      </c>
+      <c r="G239" s="12" t="inlineStr">
+        <is>
+          <t>72.6 KB</t>
+        </is>
+      </c>
+      <c r="H239" s="15" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="I239" s="16" t="inlineStr">
+        <is>
+          <t>Primary Municipal Records &amp; Educational Architecture</t>
+        </is>
+      </c>
+      <c r="J239" s="16" t="inlineStr">
+        <is>
+          <t>M.G.L. c. 121B; M.G.L. c. 184A; M.G.L. c. 44, § 7; Plymouth Registry Instruments</t>
+        </is>
+      </c>
+      <c r="K239" s="18" t="inlineStr">
+        <is>
+          <t>Dedicated 2-page educational guide and evidence ledger for family and community members. Page 1 provides a 1-page unspun narrative essay; Page 2 provides the companion Works Cited mapping every point to primary documents with repository file names.</t>
+        </is>
+      </c>
+      <c r="L239" s="15" t="inlineStr">
+        <is>
+          <t>Community Educational Guide &amp; Evidence Ledger (Verified)</t>
+        </is>
+      </c>
+      <c r="M239" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:27</t>
+        </is>
+      </c>
+      <c r="N239" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/01_Executive_and_Human_Documents/03_100_Beal_Street_The_True_Story_and_Evidence_v1.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="19" t="inlineStr">
+        <is>
+          <t>FL-324</t>
+        </is>
+      </c>
+      <c r="B240" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C240" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D240" s="20" t="inlineStr">
+        <is>
+          <t>04_100_Beal_Street_Town_vs_HHA_Legal_Chronology_and_Minutes_v2.md</t>
+        </is>
+      </c>
+      <c r="E240" s="19" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="F240" s="21" t="n">
+        <v>31676</v>
+      </c>
+      <c r="G240" s="22" t="inlineStr">
+        <is>
+          <t>30.9 KB</t>
+        </is>
+      </c>
+      <c r="H240" s="19" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="I240" s="20" t="inlineStr">
+        <is>
+          <t>Primary Municipal Records / Mass. Registry of Deeds</t>
+        </is>
+      </c>
+      <c r="J240" s="20" t="inlineStr">
+        <is>
+          <t>Historical M.G.L. c. 184A, § 3; M.G.L. c. 184, § 23; M.G.L. c. 121B, § 34; Book 09097 Pg 158; Book 51379 Pg 244</t>
+        </is>
+      </c>
+      <c r="K240" s="23" t="inlineStr">
+        <is>
+          <t>Preliminary primary-source research chronology and record index; strictly neutral factual reporting; segregates verified facts, factual inferences, and open legal questions; includes missing documents inventory and disclaimer. Not a title opinion.</t>
+        </is>
+      </c>
+      <c r="L240" s="19" t="inlineStr">
+        <is>
+          <t>Neutral Primary Source Research Index &amp; Inventory (Verified)</t>
+        </is>
+      </c>
+      <c r="M240" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-17 09:44</t>
+        </is>
+      </c>
+      <c r="N240" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/01_Executive_and_Human_Documents/04_100_Beal_Street_Town_vs_HHA_Legal_Chronology_and_Minutes_v2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="15" t="inlineStr">
+        <is>
+          <t>FL-325</t>
+        </is>
+      </c>
+      <c r="B241" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C241" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D241" s="16" t="inlineStr">
+        <is>
+          <t>04_100_Beal_Street_Town_vs_HHA_Legal_Chronology_and_Minutes_v2.pdf</t>
+        </is>
+      </c>
+      <c r="E241" s="15" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F241" s="17" t="n">
+        <v>119536</v>
+      </c>
+      <c r="G241" s="12" t="inlineStr">
+        <is>
+          <t>116.7 KB</t>
+        </is>
+      </c>
+      <c r="H241" s="15" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="I241" s="16" t="inlineStr">
+        <is>
+          <t>Primary Municipal Records / Mass. Registry of Deeds</t>
+        </is>
+      </c>
+      <c r="J241" s="16" t="inlineStr">
+        <is>
+          <t>Historical M.G.L. c. 184A, § 3; M.G.L. c. 184, § 23; M.G.L. c. 121B, § 34; Book 09097 Pg 158; Book 51379 Pg 244</t>
+        </is>
+      </c>
+      <c r="K241" s="18" t="inlineStr">
+        <is>
+          <t>Preliminary primary-source research chronology and record index; strictly neutral factual reporting; segregates verified facts, factual inferences, and open legal questions; includes missing documents inventory and disclaimer. Not a title opinion.</t>
+        </is>
+      </c>
+      <c r="L241" s="15" t="inlineStr">
+        <is>
+          <t>Neutral Primary Source Research Index &amp; Inventory (Verified)</t>
+        </is>
+      </c>
+      <c r="M241" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-17 09:44</t>
+        </is>
+      </c>
+      <c r="N241" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/01_Executive_and_Human_Documents/04_100_Beal_Street_Town_vs_HHA_Legal_Chronology_and_Minutes_v2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="19" t="inlineStr">
+        <is>
+          <t>FL-326</t>
+        </is>
+      </c>
+      <c r="B242" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C242" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D242" s="20" t="inlineStr">
+        <is>
+          <t>Exhibit_01_1989_Fee_Deed_and_ZBA_Decision_Bk09097_Pg158.pdf</t>
+        </is>
+      </c>
+      <c r="E242" s="19" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F242" s="21" t="n">
+        <v>228302</v>
+      </c>
+      <c r="G242" s="22" t="inlineStr">
+        <is>
+          <t>223.0 KB</t>
+        </is>
+      </c>
+      <c r="H242" s="19" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I242" s="20" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J242" s="20" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K242" s="23" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L242" s="19" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M242" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-14 09:24</t>
+        </is>
+      </c>
+      <c r="N242" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_01_1989_Fee_Deed_and_ZBA_Decision_Bk09097_Pg158.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="15" t="inlineStr">
+        <is>
+          <t>FL-327</t>
+        </is>
+      </c>
+      <c r="B243" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C243" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D243" s="16" t="inlineStr">
+        <is>
+          <t>Exhibit_02_2001_Gale_Subdivision_Plan_and_2024_ALTA_Survey.pdf</t>
+        </is>
+      </c>
+      <c r="E243" s="15" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F243" s="17" t="n">
+        <v>2390635</v>
+      </c>
+      <c r="G243" s="12" t="inlineStr">
+        <is>
+          <t>2.3 MB</t>
+        </is>
+      </c>
+      <c r="H243" s="15" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I243" s="16" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J243" s="16" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K243" s="18" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L243" s="15" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M243" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14 09:24</t>
+        </is>
+      </c>
+      <c r="N243" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_02_2001_Gale_Subdivision_Plan_and_2024_ALTA_Survey.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="19" t="inlineStr">
+        <is>
+          <t>FL-328</t>
+        </is>
+      </c>
+      <c r="B244" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C244" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D244" s="20" t="inlineStr">
+        <is>
+          <t>Exhibit_03_2006_Town_Meeting_Article_38_Certified_Vote.pdf</t>
+        </is>
+      </c>
+      <c r="E244" s="19" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F244" s="21" t="n">
+        <v>217985</v>
+      </c>
+      <c r="G244" s="22" t="inlineStr">
+        <is>
+          <t>212.9 KB</t>
+        </is>
+      </c>
+      <c r="H244" s="19" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I244" s="20" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J244" s="20" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K244" s="23" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L244" s="19" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M244" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-14 09:24</t>
+        </is>
+      </c>
+      <c r="N244" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_03_2006_Town_Meeting_Article_38_Certified_Vote.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="15" t="inlineStr">
+        <is>
+          <t>FL-329</t>
+        </is>
+      </c>
+      <c r="B245" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C245" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D245" s="16" t="inlineStr">
+        <is>
+          <t>Exhibit_04_2019_Select_Board_Executive_Session_Minutes_Lawsuit_Vote.pdf</t>
+        </is>
+      </c>
+      <c r="E245" s="15" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F245" s="17" t="n">
+        <v>50677</v>
+      </c>
+      <c r="G245" s="12" t="inlineStr">
+        <is>
+          <t>49.5 KB</t>
+        </is>
+      </c>
+      <c r="H245" s="15" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I245" s="16" t="inlineStr">
+        <is>
+          <t>Hingham Board of Selectmen (Healey, Power, Johnson)</t>
+        </is>
+      </c>
+      <c r="J245" s="16" t="inlineStr">
+        <is>
+          <t>M.G.L. c. 30A, § 21(a)(3) (Executive Session Litigation)</t>
+        </is>
+      </c>
+      <c r="K245" s="18" t="inlineStr">
+        <is>
+          <t>Executive Session minutes of Feb 26, 2019 recording 3-0 vote to file litigation against HHA to enforce 2001 MOU 9 days before 30-yr reverter expiration.</t>
+        </is>
+      </c>
+      <c r="L245" s="15" t="inlineStr">
+        <is>
+          <t>Official Municipal Minutes (Verified)</t>
+        </is>
+      </c>
+      <c r="M245" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14 08:38</t>
+        </is>
+      </c>
+      <c r="N245" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_04_2019_Select_Board_Executive_Session_Minutes_Lawsuit_Vote.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="19" t="inlineStr">
+        <is>
+          <t>FL-330</t>
+        </is>
+      </c>
+      <c r="B246" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C246" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D246" s="20" t="inlineStr">
+        <is>
+          <t>Exhibit_05_2019_HHA_Minutes_School_Tract_II_DHCD_Intervention.pdf</t>
+        </is>
+      </c>
+      <c r="E246" s="19" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F246" s="21" t="n">
+        <v>41327</v>
+      </c>
+      <c r="G246" s="22" t="inlineStr">
+        <is>
+          <t>40.4 KB</t>
+        </is>
+      </c>
+      <c r="H246" s="19" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I246" s="20" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J246" s="20" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K246" s="23" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L246" s="19" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M246" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-14 09:13</t>
+        </is>
+      </c>
+      <c r="N246" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_05_2019_HHA_Minutes_School_Tract_II_DHCD_Intervention.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="15" t="inlineStr">
+        <is>
+          <t>FL-331</t>
+        </is>
+      </c>
+      <c r="B247" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C247" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D247" s="16" t="inlineStr">
+        <is>
+          <t>Exhibit_06_2021_HHA_Minutes_4-0_Rescission_Vote.pdf</t>
+        </is>
+      </c>
+      <c r="E247" s="15" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F247" s="17" t="n">
+        <v>101165</v>
+      </c>
+      <c r="G247" s="12" t="inlineStr">
+        <is>
+          <t>98.8 KB</t>
+        </is>
+      </c>
+      <c r="H247" s="15" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I247" s="16" t="inlineStr">
+        <is>
+          <t>Hingham Housing Authority (Dir. James Marathas)</t>
+        </is>
+      </c>
+      <c r="J247" s="16" t="inlineStr">
+        <is>
+          <t>M.G.L. c. 121B, § 34; HHA By-Laws</t>
+        </is>
+      </c>
+      <c r="K247" s="18" t="inlineStr">
+        <is>
+          <t>Official meeting minutes of Sept 7, 2021 recording 4-0 vote formally rescinding the June 5, 2019 transfer motion, keeping land in HHA ownership.</t>
+        </is>
+      </c>
+      <c r="L247" s="15" t="inlineStr">
+        <is>
+          <t>Official Board Minutes (Verified)</t>
+        </is>
+      </c>
+      <c r="M247" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:46</t>
+        </is>
+      </c>
+      <c r="N247" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_06_2021_HHA_Minutes_4-0_Rescission_Vote.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="19" t="inlineStr">
+        <is>
+          <t>FL-332</t>
+        </is>
+      </c>
+      <c r="B248" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C248" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D248" s="20" t="inlineStr">
+        <is>
+          <t>Exhibit_07_2024_MassDEP_Recorded_ORAD_Bk59527_Pg273.pdf</t>
+        </is>
+      </c>
+      <c r="E248" s="19" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F248" s="21" t="n">
+        <v>468709</v>
+      </c>
+      <c r="G248" s="22" t="inlineStr">
+        <is>
+          <t>457.7 KB</t>
+        </is>
+      </c>
+      <c r="H248" s="19" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I248" s="20" t="inlineStr">
+        <is>
+          <t>Hingham Conservation Commission / MassDEP</t>
+        </is>
+      </c>
+      <c r="J248" s="20" t="inlineStr">
+        <is>
+          <t>Plymouth County Registry of Deeds Book 59527, Page 273 (Doc #78968)</t>
+        </is>
+      </c>
+      <c r="K248" s="23" t="inlineStr">
+        <is>
+          <t>Recorded Order of Resource Area Delineation (ORAD) WPA Form 4B officially approving wetland boundary lines on Dec 10, 2024.</t>
+        </is>
+      </c>
+      <c r="L248" s="19" t="inlineStr">
+        <is>
+          <t>Recorded Order (Verified)</t>
+        </is>
+      </c>
+      <c r="M248" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-15 15:26</t>
+        </is>
+      </c>
+      <c r="N248" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_07_2024_MassDEP_Recorded_ORAD_Bk59527_Pg273.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="15" t="inlineStr">
+        <is>
+          <t>FL-333</t>
+        </is>
+      </c>
+      <c r="B249" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C249" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D249" s="16" t="inlineStr">
+        <is>
+          <t>Exhibit_08_2025_HHA_Developer_RFP_155_Pages.pdf</t>
+        </is>
+      </c>
+      <c r="E249" s="15" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F249" s="17" t="n">
+        <v>13909202</v>
+      </c>
+      <c r="G249" s="12" t="inlineStr">
+        <is>
+          <t>13.3 MB</t>
+        </is>
+      </c>
+      <c r="H249" s="15" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I249" s="16" t="inlineStr">
+        <is>
+          <t>Hingham Housing Authority (James Marathas, ED)</t>
+        </is>
+      </c>
+      <c r="J249" s="16" t="inlineStr">
+        <is>
+          <t>M.G.L. c. 30B, § 16; M.G.L. c. 121B</t>
+        </is>
+      </c>
+      <c r="K249" s="18" t="inlineStr">
+        <is>
+          <t>Official 155-page Developer RFP package including Bohler engineering study, Lucas wetlands report, Control Point boundary survey, and draft 99-year ground lease.</t>
+        </is>
+      </c>
+      <c r="L249" s="15" t="inlineStr">
+        <is>
+          <t>Authentic Public RFP (Verified)</t>
+        </is>
+      </c>
+      <c r="M249" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14 09:20</t>
+        </is>
+      </c>
+      <c r="N249" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_08_2025_HHA_Developer_RFP_155_Pages.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="19" t="inlineStr">
+        <is>
+          <t>FL-334</t>
+        </is>
+      </c>
+      <c r="B250" s="20" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C250" s="20" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D250" s="20" t="inlineStr">
+        <is>
+          <t>Exhibit_09_2025_HHA_Minutes_Peabody_Developer_Award_Vote.pdf</t>
+        </is>
+      </c>
+      <c r="E250" s="19" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F250" s="21" t="n">
+        <v>107708</v>
+      </c>
+      <c r="G250" s="22" t="inlineStr">
+        <is>
+          <t>105.2 KB</t>
+        </is>
+      </c>
+      <c r="H250" s="19" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I250" s="20" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J250" s="20" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K250" s="23" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L250" s="19" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M250" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:46</t>
+        </is>
+      </c>
+      <c r="N250" s="20" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_09_2025_HHA_Minutes_Peabody_Developer_Award_Vote.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="15" t="inlineStr">
+        <is>
+          <t>FL-335</t>
+        </is>
+      </c>
+      <c r="B251" s="16" t="inlineStr">
+        <is>
+          <t>Agent-Created Deliverable</t>
+        </is>
+      </c>
+      <c r="C251" s="16" t="inlineStr">
+        <is>
+          <t>Agent Synthesized Work</t>
+        </is>
+      </c>
+      <c r="D251" s="16" t="inlineStr">
+        <is>
+          <t>Exhibit_10_2026_Town_Meeting_Warrant_Article_12_CAL_Debt_Defeat.pdf</t>
+        </is>
+      </c>
+      <c r="E251" s="15" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="F251" s="17" t="n">
+        <v>2958699</v>
+      </c>
+      <c r="G251" s="12" t="inlineStr">
+        <is>
+          <t>2.8 MB</t>
+        </is>
+      </c>
+      <c r="H251" s="15" t="inlineStr">
+        <is>
+          <t>Original Public Record</t>
+        </is>
+      </c>
+      <c r="I251" s="16" t="inlineStr">
+        <is>
+          <t>Town of Hingham / Housing Authority</t>
+        </is>
+      </c>
+      <c r="J251" s="16" t="inlineStr">
+        <is>
+          <t>Massachusetts General Laws</t>
+        </is>
+      </c>
+      <c r="K251" s="18" t="inlineStr">
+        <is>
+          <t>Project documentation and archival record.</t>
+        </is>
+      </c>
+      <c r="L251" s="15" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M251" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14 09:19</t>
+        </is>
+      </c>
+      <c r="N251" s="16" t="inlineStr">
+        <is>
+          <t>agent_created_deliverables/packages/100_Beal_Street_Verifiable_Facts_and_Evidence_Package_v1/02_Primary_Source_Evidence_Exhibits/Exhibit_10_2026_Town_Meeting_Warrant_Article_12_CAL_Debt_Defeat.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:N231"/>
+  <autoFilter ref="A4:N251"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>